<commit_message>
Update Week 1 QA testing documents
</commit_message>
<xml_diff>
--- a/Week1/04-RTM/Requirements_Traceability_Matrix.xlsx
+++ b/Week1/04-RTM/Requirements_Traceability_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2d058293596cab1/Desktop/Software-QA-Tester/Week1/04-RTM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F25DC773A252ABDACC10480651DF61A45BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CA6FD6C-9C4C-4341-813E-1243AED36B5A}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_F25DC773A252ABDACC10480651DF61A45BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E80A594-D59F-452B-9C24-0823C7DD87D9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="61">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Test Status</t>
   </si>
   <si>
-    <t>Bug ID</t>
-  </si>
-  <si>
     <t>REQ-001</t>
   </si>
   <si>
@@ -66,15 +63,9 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>REQ-002</t>
   </si>
   <si>
-    <t>User should be able to view the correct product image</t>
-  </si>
-  <si>
     <t>TC-PROD-001</t>
   </si>
   <si>
@@ -84,9 +75,6 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>BUG-001</t>
-  </si>
-  <si>
     <t>REQ-003</t>
   </si>
   <si>
@@ -99,30 +87,18 @@
     <t>Verify Add to Cart functionality</t>
   </si>
   <si>
-    <t>BUG-002</t>
-  </si>
-  <si>
     <t>REQ-004</t>
   </si>
   <si>
-    <t>User should be able to enter Last Name during checkout</t>
-  </si>
-  <si>
     <t>TC-CHECKOUT-001</t>
   </si>
   <si>
     <t>Verify Last Name field accepts text</t>
   </si>
   <si>
-    <t>BUG-003</t>
-  </si>
-  <si>
     <t>REQ-005</t>
   </si>
   <si>
-    <t>User should be able to sort products by price</t>
-  </si>
-  <si>
     <t>TC-PROD-002</t>
   </si>
   <si>
@@ -132,30 +108,18 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>BUG-004</t>
-  </si>
-  <si>
     <t>REQ-006</t>
   </si>
   <si>
-    <t>User should be able to remove a product from cart</t>
-  </si>
-  <si>
     <t>TC-CART-002</t>
   </si>
   <si>
     <t>Verify Remove button functionality</t>
   </si>
   <si>
-    <t>BUG-005</t>
-  </si>
-  <si>
     <t>REQ-007</t>
   </si>
   <si>
-    <t>User should be able to proceed to checkout with products in cart</t>
-  </si>
-  <si>
     <t>TC-CHECKOUT-002</t>
   </si>
   <si>
@@ -177,9 +141,6 @@
     <t>REQ-009</t>
   </si>
   <si>
-    <t>User should be able to review selected products before checkout</t>
-  </si>
-  <si>
     <t>TC-CART-003</t>
   </si>
   <si>
@@ -202,13 +163,58 @@
   </si>
   <si>
     <t>Not Executed</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Requirement Type</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Correct product image should be displayed</t>
+  </si>
+  <si>
+    <t>Shopping Cart</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>User should be able to enter Last Name</t>
+  </si>
+  <si>
+    <t>Product Sorting</t>
+  </si>
+  <si>
+    <t>Products should be sorted according to selected order</t>
+  </si>
+  <si>
+    <t>User should be able to remove a product</t>
+  </si>
+  <si>
+    <t>User should be able to proceed to checkout</t>
+  </si>
+  <si>
+    <t>User should be able to review selected products</t>
+  </si>
+  <si>
+    <t>Order</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +274,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -533,266 +543,301 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="33" customWidth="1"/>
+    <col min="1" max="1" width="28.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="43.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="86.4">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="72">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:8" ht="72">
+      <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="86.4">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="57.6">
+      <c r="A6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="72">
+      <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="57.6">
+      <c r="A8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="2" t="s">
+    </row>
+    <row r="9" spans="1:8" ht="57.6">
+      <c r="A9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="G9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="72">
+      <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="2" t="s">
+      <c r="G10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="72">
+      <c r="A11" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>